<commit_message>
Stage 8 review fixes: A-019
</commit_message>
<xml_diff>
--- a/output/archive/VellacombeData/Clients/NLM/VD-26-091/Routes/Scout/NLM-A_boronate_21Aug26_v2.xlsx
+++ b/output/archive/VellacombeData/Clients/NLM/VD-26-091/Routes/Scout/NLM-A_boronate_21Aug26_v2.xlsx
@@ -60,13 +60,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -164,9 +162,9 @@
     <author>Hassan Darwish</author>
   </authors>
   <commentList>
-    <comment ref="F3" authorId="0" shapeId="0">
+    <comment ref="C2" authorId="0" shapeId="0">
       <text>
-        <t>LCMS trace is in the project folder. Protodeboronation product is clearly visible in the trace.</t>
+        <t>Refer to the route scout records for attempt details; analytical interpretation is not transcribed here.</t>
       </text>
     </comment>
   </commentList>
@@ -181,7 +179,7 @@
   <commentList>
     <comment ref="D2" authorId="0" shapeId="0">
       <text>
-        <t>Client asked for a view by the end of the month. Chase on Monday if nothing by then.</t>
+        <t>Decision timing still to be confirmed with the client.</t>
       </text>
     </comment>
   </commentList>
@@ -581,7 +579,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>The unstable boronate has stopped the route scout. The team is evaluating a protected alternative with the client. Start date and batch size depend on the client's answer [TBC].</t>
+          <t>The unstable boronate has delayed the route scout, which started on 20 Jul 2026. The team is evaluating a protected alternative with the client. Timing and scope of further work remain [TBC].</t>
         </is>
       </c>
     </row>
@@ -614,50 +612,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="46" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Attempt</t>
+          <t>Record</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Boronate form</t>
+          <t>Route issue</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Protecting group</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Conditions</t>
+          <t>Scale (mg)</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Scale (mg)</t>
+          <t>Outcome</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Outcome</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Next step</t>
         </is>
@@ -666,170 +658,63 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>A-01</t>
+          <t>Boronate route scout</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Free boronic acid</t>
+          <t>Unstable boronate</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Suzuki partner, aqueous base, 80 °C</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n">
-        <v>200</v>
+          <t>See route scout records</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Route scout delayed</t>
+        </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Decomposed on standing; protodeboronation seen by LCMS</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Stop; do not repeat</t>
+          <t>Evaluate protected alternative with client</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A-02</t>
+          <t>Protected alternative</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Free boronic acid</t>
+          <t>Under evaluation</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Same, degassed solvents, 60 °C</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>200</v>
-      </c>
+          <t>[TBC]</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Await LCMS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>A-03</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Pinacol ester</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Pinacol</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Suzuki partner, carbonate base, 80 °C</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Queued</t>
-        </is>
-      </c>
-    </row>
+          <t>Client decision pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>A-04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>MIDA boronate</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>MIDA</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Slow release, aqueous base, 60 °C</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>100</v>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>A-05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Trifluoroborate</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Potassium salt</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="4" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="E7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="4" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="E9" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -889,7 +774,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Pinacol / MIDA / trifluoroborate</t>
+          <t>Protected alternative [TBC]</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -911,12 +796,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Accept the slower route if it gives a stable intermediate</t>
+          <t>Agree route implications of protected alternative</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Yes / no</t>
+          <t>[TBC]</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -961,7 +846,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Change of order: attempt a different building block</t>
+          <t>Confirm further scout scope</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -977,7 +862,7 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Open</t>
         </is>
       </c>
     </row>

</xml_diff>